<commit_message>
Add JSON files for data management and sharing plans
- Created sample1.json for the llama3.1-8b_pdfplumber_rda output, detailing a data management and sharing plan with contact information, datasets, and ethical considerations.
- Created sample1.json for the merged gemma4-e4b+llama3.1-8b_pdfplumber output, including a comprehensive narrative section with detailed responses to data management elements, such as data types, preservation, access, and oversight.
</commit_message>
<xml_diff>
--- a/data/output/5_rda/llama3.1-8b_pdfplumber_rda/evaluation/evaluation_results.xlsx
+++ b/data/output/5_rda/llama3.1-8b_pdfplumber_rda/evaluation/evaluation_results.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="108">
   <si>
     <t>model</t>
   </si>
@@ -76,25 +76,109 @@
     <t>dmp.dataset[0].distribution[0].host.title</t>
   </si>
   <si>
+    <t>dmp.dataset[0].title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].description</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[0].host.title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[1].host.title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[1].title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].description</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].distribution[0].host.title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].title</t>
+  </si>
+  <si>
+    <t>dmp.title</t>
+  </si>
+  <si>
+    <t>Dataset description</t>
+  </si>
+  <si>
+    <t>Storage place (host)</t>
+  </si>
+  <si>
+    <t>Dataset title</t>
+  </si>
+  <si>
+    <t>Other distribution details</t>
+  </si>
+  <si>
+    <t>Plan title &amp; description</t>
+  </si>
+  <si>
+    <t>Missed</t>
+  </si>
+  <si>
+    <t>Mismatch</t>
+  </si>
+  <si>
+    <t>Correct</t>
+  </si>
+  <si>
+    <t>model field</t>
+  </si>
+  <si>
+    <t>model value</t>
+  </si>
+  <si>
+    <t>reference value</t>
+  </si>
+  <si>
+    <t>verdict</t>
+  </si>
+  <si>
+    <t>reason</t>
+  </si>
+  <si>
+    <t>dmp.contact.contact_id[0].identifier</t>
+  </si>
+  <si>
+    <t>dmp.contact.contact_id[0].type</t>
+  </si>
+  <si>
+    <t>dmp.contact.mbox</t>
+  </si>
+  <si>
+    <t>dmp.contact.name</t>
+  </si>
+  <si>
+    <t>dmp.created</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].dataset_id.identifier</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].dataset_id.type</t>
+  </si>
+  <si>
     <t>dmp.dataset[0].personal_data</t>
   </si>
   <si>
     <t>dmp.dataset[0].sensitive_data</t>
   </si>
   <si>
-    <t>dmp.dataset[0].title</t>
-  </si>
-  <si>
-    <t>dmp.dataset[1].description</t>
-  </si>
-  <si>
-    <t>dmp.dataset[1].metadata[0].description</t>
-  </si>
-  <si>
-    <t>dmp.dataset[1].metadata[0].language</t>
-  </si>
-  <si>
-    <t>dmp.dataset[1].metadata[1].description</t>
+    <t>dmp.dataset[0].type</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].dataset_id.identifier</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].dataset_id.type</t>
   </si>
   <si>
     <t>dmp.dataset[1].personal_data</t>
@@ -103,16 +187,13 @@
     <t>dmp.dataset[1].sensitive_data</t>
   </si>
   <si>
-    <t>dmp.dataset[1].title</t>
-  </si>
-  <si>
-    <t>dmp.dataset[2].description</t>
-  </si>
-  <si>
-    <t>dmp.dataset[2].distribution[0].license[0].license_ref</t>
-  </si>
-  <si>
-    <t>dmp.dataset[2].metadata[0].language</t>
+    <t>dmp.dataset[1].type</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].dataset_id.identifier</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].dataset_id.type</t>
   </si>
   <si>
     <t>dmp.dataset[2].personal_data</t>
@@ -121,13 +202,13 @@
     <t>dmp.dataset[2].sensitive_data</t>
   </si>
   <si>
-    <t>dmp.dataset[2].title</t>
-  </si>
-  <si>
-    <t>dmp.dataset[3].description</t>
-  </si>
-  <si>
-    <t>dmp.dataset[3].metadata[0].language</t>
+    <t>dmp.dataset[2].type</t>
+  </si>
+  <si>
+    <t>dmp.dataset[3].dataset_id.identifier</t>
+  </si>
+  <si>
+    <t>dmp.dataset[3].dataset_id.type</t>
   </si>
   <si>
     <t>dmp.dataset[3].personal_data</t>
@@ -139,94 +220,7 @@
     <t>dmp.dataset[3].title</t>
   </si>
   <si>
-    <t>dmp.description</t>
-  </si>
-  <si>
-    <t>dmp.title</t>
-  </si>
-  <si>
-    <t>Dataset description</t>
-  </si>
-  <si>
-    <t>Storage place (host)</t>
-  </si>
-  <si>
-    <t>Personal &amp; sensitive data</t>
-  </si>
-  <si>
-    <t>Dataset title</t>
-  </si>
-  <si>
-    <t>Metadata &amp; standards</t>
-  </si>
-  <si>
-    <t>Licence</t>
-  </si>
-  <si>
-    <t>Plan title &amp; description</t>
-  </si>
-  <si>
-    <t>Missed</t>
-  </si>
-  <si>
-    <t>Correct</t>
-  </si>
-  <si>
-    <t>model field</t>
-  </si>
-  <si>
-    <t>model value</t>
-  </si>
-  <si>
-    <t>reference value</t>
-  </si>
-  <si>
-    <t>verdict</t>
-  </si>
-  <si>
-    <t>reason</t>
-  </si>
-  <si>
-    <t>dmp.contact.contact_id[0].identifier</t>
-  </si>
-  <si>
-    <t>dmp.contact.contact_id[0].type</t>
-  </si>
-  <si>
-    <t>dmp.contact.mbox</t>
-  </si>
-  <si>
-    <t>dmp.contact.name</t>
-  </si>
-  <si>
-    <t>dmp.created</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].dataset_id.identifier</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].dataset_id.type</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].type</t>
-  </si>
-  <si>
-    <t>dmp.dataset[1].dataset_id.identifier</t>
-  </si>
-  <si>
-    <t>dmp.dataset[1].dataset_id.type</t>
-  </si>
-  <si>
-    <t>dmp.dataset[1].type</t>
-  </si>
-  <si>
-    <t>dmp.dataset[2].dataset_id.identifier</t>
-  </si>
-  <si>
-    <t>dmp.dataset[2].dataset_id.type</t>
-  </si>
-  <si>
-    <t>dmp.dataset[2].type</t>
+    <t>dmp.dataset[3].type</t>
   </si>
   <si>
     <t>dmp.dmp_id.identifier</t>
@@ -244,28 +238,55 @@
     <t>dmp.modified</t>
   </si>
   <si>
-    <t>0000-0003-0644-4174</t>
+    <t>https://orcid.org/0000-0003-0644-4174</t>
   </si>
   <si>
     <t>orcid</t>
   </si>
   <si>
+    <t>john.doe@example.com</t>
+  </si>
+  <si>
+    <t>John Doe</t>
+  </si>
+  <si>
     <t>2026-10-19T00:00:00Z</t>
   </si>
   <si>
+    <t>https://example.com/dataset</t>
+  </si>
+  <si>
+    <t>url</t>
+  </si>
+  <si>
     <t>no</t>
   </si>
   <si>
-    <t>Data related to each of our proposed experiments</t>
+    <t>Secondary data analysis project</t>
   </si>
   <si>
     <t>dataset</t>
   </si>
   <si>
-    <t>Code and results for all analyses completed on experimental data</t>
-  </si>
-  <si>
-    <t>Simulation code for controller development and testing</t>
+    <t>https://example.com/dataset2</t>
+  </si>
+  <si>
+    <t>RISE study</t>
+  </si>
+  <si>
+    <t>https://example.com/dataset3</t>
+  </si>
+  <si>
+    <t>iWATCH study</t>
+  </si>
+  <si>
+    <t>https://example.com/dataset4</t>
+  </si>
+  <si>
+    <t>NHANES cohorts</t>
+  </si>
+  <si>
+    <t>https://example.com/dmp</t>
   </si>
   <si>
     <t>unknown</t>
@@ -274,49 +295,40 @@
     <t>eng</t>
   </si>
   <si>
-    <t>CPS 2015</t>
+    <t>DATA MANAGEMENT AND SHARING PLAN</t>
   </si>
   <si>
     <t>None</t>
   </si>
   <si>
-    <t>data related to each of our proposed experiments</t>
-  </si>
-  <si>
-    <t>code and results for all analyses completed on experimental data</t>
-  </si>
-  <si>
-    <t>simulation code for controller development and testing</t>
-  </si>
-  <si>
-    <t>First, we will have data related to each of our proposed experiments. These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session.</t>
-  </si>
-  <si>
-    <t>servers at the Rehabilitation Institute of Chicago</t>
-  </si>
-  <si>
-    <t>Our second type of data will be the code and results for all analyses completed on experimental data. Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts.</t>
-  </si>
-  <si>
-    <t>The contents of each data file, including the experimental conditions or the analysis procedures used during generation will be documented.</t>
-  </si>
-  <si>
-    <t>The code needed to generate all published results will be documented clearly.</t>
-  </si>
-  <si>
-    <t>The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
-  </si>
-  <si>
-    <t>GNU Public License</t>
-  </si>
-  <si>
-    <t>Select videos of the experiments will be distributed, with subject faces blurred so as to be unidentifiable.</t>
-  </si>
-  <si>
-    <t>videos of the experiments</t>
-  </si>
-  <si>
-    <t>We will manage all scientific and technical content generated from this proposal. Our products will include 3 broad types of data.</t>
+    <t>Objective sedentary behavior metrics</t>
+  </si>
+  <si>
+    <t>custom code and models</t>
+  </si>
+  <si>
+    <t>study protocols</t>
+  </si>
+  <si>
+    <t>As this is a secondary data analysis project, we will only be able to publicly share in the UC San Diego Library Repository sitting behavior metrics or analysis that were created in this project from the following UCSD-based study datasets: (i) The RISE study (ii) The iWATCH study (iii) NHANES cohorts</t>
+  </si>
+  <si>
+    <t>University of California San Diego Library repository</t>
+  </si>
+  <si>
+    <t>All custom code and models will also be shared in the data repository and on our project's GitHub website, hosted as part of the UCSD Advance Data Analytics Lab GitHub and titled "Deep Postures".</t>
+  </si>
+  <si>
+    <t>UCSD Advance Data Analytics Lab GitHub</t>
+  </si>
+  <si>
+    <t>Deep Postures</t>
+  </si>
+  <si>
+    <t>It will be deposited into the UC San Diego Library Data repository along with study protocols, code, and models for public use.</t>
+  </si>
+  <si>
+    <t>UC San Diego Library Data repository</t>
   </si>
   <si>
     <t>Hallucinated</t>
@@ -325,14 +337,17 @@
     <t>not in the reference</t>
   </si>
   <si>
-    <t>both empty</t>
+    <t>only 0% of the model's words are in the reference</t>
+  </si>
+  <si>
+    <t>only 50% of the model's words are in the reference</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -347,6 +362,13 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -381,16 +403,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -726,28 +754,28 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="E2">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="G2">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="H2">
-        <v>0.6899999999999999</v>
+        <v>0.029</v>
       </c>
       <c r="I2">
-        <v>0.4</v>
+        <v>0.083</v>
       </c>
       <c r="J2">
-        <v>0.506</v>
+        <v>0.043</v>
       </c>
     </row>
   </sheetData>
@@ -797,37 +825,37 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>12</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
         <v>3</v>
       </c>
-      <c r="B2">
-        <v>25</v>
-      </c>
-      <c r="C2">
-        <v>20</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
       <c r="E2">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F2">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="G2">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="H2">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="I2">
-        <v>0.6899999999999999</v>
+        <v>0.029</v>
       </c>
       <c r="J2">
-        <v>0.4</v>
+        <v>0.083</v>
       </c>
       <c r="K2">
-        <v>0.506</v>
+        <v>0.043</v>
       </c>
     </row>
   </sheetData>
@@ -837,7 +865,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -856,352 +884,170 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="D2" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
         <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="D3" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B4" t="s">
         <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="D4" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B5" t="s">
         <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B6" t="s">
         <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="D6" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B7" t="s">
         <v>22</v>
       </c>
       <c r="C7" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="D7" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
         <v>23</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="D8" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B9" t="s">
         <v>24</v>
       </c>
       <c r="C9" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B10" t="s">
         <v>25</v>
       </c>
       <c r="C10" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="D10" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B11" t="s">
         <v>26</v>
       </c>
       <c r="C11" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="D11" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B12" t="s">
         <v>27</v>
       </c>
       <c r="C12" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="D12" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B13" t="s">
         <v>28</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="D13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15">
-        <v>3</v>
-      </c>
-      <c r="B15" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" t="s">
-        <v>47</v>
-      </c>
-      <c r="D15" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16">
-        <v>3</v>
-      </c>
-      <c r="B16" t="s">
-        <v>31</v>
-      </c>
-      <c r="C16" t="s">
-        <v>46</v>
-      </c>
-      <c r="D16" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17">
-        <v>3</v>
-      </c>
-      <c r="B17" t="s">
-        <v>32</v>
-      </c>
-      <c r="C17" t="s">
-        <v>44</v>
-      </c>
-      <c r="D17" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18">
-        <v>3</v>
-      </c>
-      <c r="B18" t="s">
-        <v>33</v>
-      </c>
-      <c r="C18" t="s">
-        <v>44</v>
-      </c>
-      <c r="D18" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19">
-        <v>3</v>
-      </c>
-      <c r="B19" t="s">
-        <v>34</v>
-      </c>
-      <c r="C19" t="s">
-        <v>45</v>
-      </c>
-      <c r="D19" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="A20">
-        <v>3</v>
-      </c>
-      <c r="B20" t="s">
-        <v>35</v>
-      </c>
-      <c r="C20" t="s">
-        <v>42</v>
-      </c>
-      <c r="D20" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4">
-      <c r="A21">
-        <v>3</v>
-      </c>
-      <c r="B21" t="s">
         <v>36</v>
-      </c>
-      <c r="C21" t="s">
-        <v>46</v>
-      </c>
-      <c r="D21" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4">
-      <c r="A22">
-        <v>3</v>
-      </c>
-      <c r="B22" t="s">
-        <v>37</v>
-      </c>
-      <c r="C22" t="s">
-        <v>44</v>
-      </c>
-      <c r="D22" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
-      <c r="A23">
-        <v>3</v>
-      </c>
-      <c r="B23" t="s">
-        <v>38</v>
-      </c>
-      <c r="C23" t="s">
-        <v>44</v>
-      </c>
-      <c r="D23" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4">
-      <c r="A24">
-        <v>3</v>
-      </c>
-      <c r="B24" t="s">
-        <v>39</v>
-      </c>
-      <c r="C24" t="s">
-        <v>45</v>
-      </c>
-      <c r="D24" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4">
-      <c r="A25">
-        <v>3</v>
-      </c>
-      <c r="B25" t="s">
-        <v>40</v>
-      </c>
-      <c r="C25" t="s">
-        <v>48</v>
-      </c>
-      <c r="D25" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4">
-      <c r="A26">
-        <v>3</v>
-      </c>
-      <c r="B26" t="s">
-        <v>41</v>
-      </c>
-      <c r="C26" t="s">
-        <v>48</v>
-      </c>
-      <c r="D26" t="s">
-        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1211,7 +1057,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1222,884 +1068,1019 @@
         <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="C2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D2" t="s">
-        <v>75</v>
+        <v>42</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>73</v>
       </c>
       <c r="E2" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F2" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="G2" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="C3" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E3" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F3" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="G3" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>44</v>
+      </c>
+      <c r="D4" t="s">
+        <v>75</v>
       </c>
       <c r="E4" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F4" t="s">
-        <v>50</v>
+        <v>104</v>
       </c>
       <c r="G4" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C5" t="s">
-        <v>59</v>
+        <v>45</v>
+      </c>
+      <c r="D5" t="s">
+        <v>76</v>
       </c>
       <c r="E5" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F5" t="s">
-        <v>50</v>
+        <v>104</v>
       </c>
       <c r="G5" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="D6" t="s">
         <v>77</v>
       </c>
       <c r="E6" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F6" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="G6" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="C7" t="s">
-        <v>61</v>
+        <v>47</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>78</v>
       </c>
       <c r="E7" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F7" t="s">
-        <v>50</v>
+        <v>104</v>
       </c>
       <c r="G7" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="C8" t="s">
-        <v>62</v>
+        <v>48</v>
+      </c>
+      <c r="D8" t="s">
+        <v>79</v>
       </c>
       <c r="E8" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F8" t="s">
-        <v>50</v>
+        <v>104</v>
       </c>
       <c r="G8" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="C9" t="s">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="D9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E9" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="F9" t="s">
-        <v>50</v>
+        <v>104</v>
+      </c>
+      <c r="G9" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="C10" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="D10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E10" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="F10" t="s">
-        <v>50</v>
+        <v>104</v>
+      </c>
+      <c r="G10" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E11" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="F11" t="s">
-        <v>50</v>
+        <v>104</v>
+      </c>
+      <c r="G11" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="C12" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="D12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E12" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F12" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="G12" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B13" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="C13" t="s">
-        <v>64</v>
+        <v>52</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>83</v>
       </c>
       <c r="E13" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F13" t="s">
-        <v>50</v>
+        <v>104</v>
       </c>
       <c r="G13" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="C14" t="s">
-        <v>65</v>
+        <v>53</v>
+      </c>
+      <c r="D14" t="s">
+        <v>79</v>
       </c>
       <c r="E14" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F14" t="s">
-        <v>50</v>
+        <v>104</v>
       </c>
       <c r="G14" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>26</v>
+        <v>54</v>
       </c>
       <c r="C15" t="s">
-        <v>26</v>
+        <v>54</v>
       </c>
       <c r="D15" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E15" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="F15" t="s">
-        <v>50</v>
+        <v>104</v>
+      </c>
+      <c r="G15" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B16" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="C16" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="D16" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E16" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="F16" t="s">
-        <v>50</v>
+        <v>104</v>
+      </c>
+      <c r="G16" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B17" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C17" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D17" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="E17" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="F17" t="s">
-        <v>50</v>
+        <v>104</v>
+      </c>
+      <c r="G17" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B18" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="C18" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="D18" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E18" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F18" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="G18" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B19" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C19" t="s">
-        <v>67</v>
+        <v>57</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>85</v>
       </c>
       <c r="E19" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F19" t="s">
-        <v>50</v>
+        <v>104</v>
       </c>
       <c r="G19" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B20" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="C20" t="s">
-        <v>68</v>
+        <v>58</v>
+      </c>
+      <c r="D20" t="s">
+        <v>79</v>
       </c>
       <c r="E20" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F20" t="s">
-        <v>50</v>
+        <v>104</v>
       </c>
       <c r="G20" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B21" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="C21" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="D21" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E21" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="F21" t="s">
-        <v>50</v>
+        <v>104</v>
+      </c>
+      <c r="G21" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="C22" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="D22" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E22" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="F22" t="s">
-        <v>50</v>
+        <v>104</v>
+      </c>
+      <c r="G22" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B23" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="C23" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="D23" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="E23" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="F23" t="s">
-        <v>50</v>
+        <v>104</v>
+      </c>
+      <c r="G23" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B24" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="C24" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="D24" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E24" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F24" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="G24" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B25" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="C25" t="s">
-        <v>70</v>
+        <v>62</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>87</v>
       </c>
       <c r="E25" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F25" t="s">
-        <v>50</v>
+        <v>104</v>
       </c>
       <c r="G25" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="26" spans="1:7">
       <c r="A26">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B26" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="C26" t="s">
-        <v>71</v>
+        <v>63</v>
+      </c>
+      <c r="D26" t="s">
+        <v>79</v>
       </c>
       <c r="E26" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F26" t="s">
-        <v>50</v>
+        <v>104</v>
       </c>
       <c r="G26" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="27" spans="1:7">
       <c r="A27">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B27" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="C27" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="D27" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E27" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F27" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="G27" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="28" spans="1:7">
       <c r="A28">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B28" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="C28" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="D28" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="E28" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F28" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="G28" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="29" spans="1:7">
       <c r="A29">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B29" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="C29" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="D29" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="E29" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F29" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="G29" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="30" spans="1:7">
       <c r="A30">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B30" t="s">
-        <v>41</v>
+        <v>67</v>
       </c>
       <c r="C30" t="s">
-        <v>41</v>
+        <v>67</v>
       </c>
       <c r="D30" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="E30" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="F30" t="s">
-        <v>50</v>
+        <v>104</v>
+      </c>
+      <c r="G30" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="31" spans="1:7">
       <c r="A31">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B31" t="s">
-        <v>17</v>
-      </c>
-      <c r="D31" t="s">
-        <v>86</v>
+        <v>68</v>
+      </c>
+      <c r="C31" t="s">
+        <v>68</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>89</v>
       </c>
       <c r="E31" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F31" t="s">
-        <v>49</v>
+        <v>104</v>
+      </c>
+      <c r="G31" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="32" spans="1:7">
       <c r="A32">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B32" t="s">
+        <v>69</v>
+      </c>
+      <c r="C32" t="s">
+        <v>69</v>
+      </c>
+      <c r="D32" t="s">
+        <v>79</v>
+      </c>
+      <c r="E32" t="s">
+        <v>93</v>
+      </c>
+      <c r="F32" t="s">
+        <v>104</v>
+      </c>
+      <c r="G32" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33">
+        <v>1</v>
+      </c>
+      <c r="B33" t="s">
+        <v>70</v>
+      </c>
+      <c r="C33" t="s">
+        <v>70</v>
+      </c>
+      <c r="D33" t="s">
+        <v>90</v>
+      </c>
+      <c r="E33" t="s">
+        <v>93</v>
+      </c>
+      <c r="F33" t="s">
+        <v>104</v>
+      </c>
+      <c r="G33" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34">
+        <v>1</v>
+      </c>
+      <c r="B34" t="s">
+        <v>71</v>
+      </c>
+      <c r="C34" t="s">
+        <v>71</v>
+      </c>
+      <c r="D34" t="s">
+        <v>91</v>
+      </c>
+      <c r="E34" t="s">
+        <v>93</v>
+      </c>
+      <c r="F34" t="s">
+        <v>104</v>
+      </c>
+      <c r="G34" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35">
+        <v>1</v>
+      </c>
+      <c r="B35" t="s">
+        <v>72</v>
+      </c>
+      <c r="C35" t="s">
+        <v>72</v>
+      </c>
+      <c r="D35" t="s">
+        <v>77</v>
+      </c>
+      <c r="E35" t="s">
+        <v>93</v>
+      </c>
+      <c r="F35" t="s">
+        <v>104</v>
+      </c>
+      <c r="G35" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36">
+        <v>1</v>
+      </c>
+      <c r="B36" t="s">
+        <v>28</v>
+      </c>
+      <c r="C36" t="s">
+        <v>28</v>
+      </c>
+      <c r="D36" t="s">
+        <v>92</v>
+      </c>
+      <c r="E36" t="s">
+        <v>92</v>
+      </c>
+      <c r="F36" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37">
+        <v>1</v>
+      </c>
+      <c r="B37" t="s">
+        <v>17</v>
+      </c>
+      <c r="D37" t="s">
+        <v>93</v>
+      </c>
+      <c r="E37" t="s">
+        <v>97</v>
+      </c>
+      <c r="F37" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38">
+        <v>1</v>
+      </c>
+      <c r="B38" t="s">
         <v>18</v>
       </c>
-      <c r="D32" t="s">
-        <v>86</v>
-      </c>
-      <c r="E32" t="s">
-        <v>91</v>
-      </c>
-      <c r="F32" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6">
-      <c r="A33">
-        <v>3</v>
-      </c>
-      <c r="B33" t="s">
+      <c r="D38" t="s">
+        <v>93</v>
+      </c>
+      <c r="E38" t="s">
+        <v>98</v>
+      </c>
+      <c r="F38" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39">
+        <v>1</v>
+      </c>
+      <c r="B39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D39" t="s">
+        <v>93</v>
+      </c>
+      <c r="E39" t="s">
+        <v>94</v>
+      </c>
+      <c r="F39" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40">
+        <v>1</v>
+      </c>
+      <c r="B40" t="s">
+        <v>20</v>
+      </c>
+      <c r="D40" t="s">
+        <v>93</v>
+      </c>
+      <c r="E40" t="s">
+        <v>99</v>
+      </c>
+      <c r="F40" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41">
+        <v>1</v>
+      </c>
+      <c r="B41" t="s">
+        <v>21</v>
+      </c>
+      <c r="D41" t="s">
+        <v>93</v>
+      </c>
+      <c r="E41" t="s">
+        <v>98</v>
+      </c>
+      <c r="F41" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42">
+        <v>1</v>
+      </c>
+      <c r="B42" t="s">
         <v>22</v>
       </c>
-      <c r="D33" t="s">
-        <v>86</v>
-      </c>
-      <c r="E33" t="s">
-        <v>92</v>
-      </c>
-      <c r="F33" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6">
-      <c r="A34">
-        <v>3</v>
-      </c>
-      <c r="B34" t="s">
+      <c r="D42" t="s">
+        <v>93</v>
+      </c>
+      <c r="E42" t="s">
+        <v>100</v>
+      </c>
+      <c r="F42" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
+      <c r="A43">
+        <v>1</v>
+      </c>
+      <c r="B43" t="s">
         <v>23</v>
       </c>
-      <c r="D34" t="s">
-        <v>86</v>
-      </c>
-      <c r="E34" t="s">
-        <v>93</v>
-      </c>
-      <c r="F34" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6">
-      <c r="A35">
-        <v>3</v>
-      </c>
-      <c r="B35" t="s">
+      <c r="D43" t="s">
+        <v>93</v>
+      </c>
+      <c r="E43" t="s">
+        <v>101</v>
+      </c>
+      <c r="F43" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
+      <c r="A44">
+        <v>1</v>
+      </c>
+      <c r="B44" t="s">
         <v>24</v>
       </c>
-      <c r="D35" t="s">
-        <v>86</v>
-      </c>
-      <c r="E35" t="s">
-        <v>84</v>
-      </c>
-      <c r="F35" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6">
-      <c r="A36">
-        <v>3</v>
-      </c>
-      <c r="B36" t="s">
+      <c r="D44" t="s">
+        <v>93</v>
+      </c>
+      <c r="E44" t="s">
+        <v>95</v>
+      </c>
+      <c r="F44" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="A45">
+        <v>1</v>
+      </c>
+      <c r="B45" t="s">
         <v>25</v>
       </c>
-      <c r="D36" t="s">
-        <v>86</v>
-      </c>
-      <c r="E36" t="s">
-        <v>94</v>
-      </c>
-      <c r="F36" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6">
-      <c r="A37">
-        <v>3</v>
-      </c>
-      <c r="B37" t="s">
-        <v>29</v>
-      </c>
-      <c r="D37" t="s">
-        <v>86</v>
-      </c>
-      <c r="E37" t="s">
-        <v>95</v>
-      </c>
-      <c r="F37" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6">
-      <c r="A38">
-        <v>3</v>
-      </c>
-      <c r="B38" t="s">
-        <v>30</v>
-      </c>
-      <c r="D38" t="s">
-        <v>86</v>
-      </c>
-      <c r="E38" t="s">
+      <c r="D45" t="s">
+        <v>93</v>
+      </c>
+      <c r="E45" t="s">
+        <v>102</v>
+      </c>
+      <c r="F45" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
+      <c r="A46">
+        <v>1</v>
+      </c>
+      <c r="B46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46" t="s">
+        <v>93</v>
+      </c>
+      <c r="E46" t="s">
+        <v>103</v>
+      </c>
+      <c r="F46" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
+      <c r="A47">
+        <v>1</v>
+      </c>
+      <c r="B47" t="s">
+        <v>27</v>
+      </c>
+      <c r="D47" t="s">
+        <v>93</v>
+      </c>
+      <c r="E47" t="s">
         <v>96</v>
       </c>
-      <c r="F38" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6">
-      <c r="A39">
-        <v>3</v>
-      </c>
-      <c r="B39" t="s">
-        <v>31</v>
-      </c>
-      <c r="D39" t="s">
-        <v>86</v>
-      </c>
-      <c r="E39" t="s">
-        <v>84</v>
-      </c>
-      <c r="F39" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6">
-      <c r="A40">
-        <v>3</v>
-      </c>
-      <c r="B40" t="s">
-        <v>35</v>
-      </c>
-      <c r="D40" t="s">
-        <v>86</v>
-      </c>
-      <c r="E40" t="s">
-        <v>97</v>
-      </c>
-      <c r="F40" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6">
-      <c r="A41">
-        <v>3</v>
-      </c>
-      <c r="B41" t="s">
-        <v>36</v>
-      </c>
-      <c r="D41" t="s">
-        <v>86</v>
-      </c>
-      <c r="E41" t="s">
-        <v>84</v>
-      </c>
-      <c r="F41" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6">
-      <c r="A42">
-        <v>3</v>
-      </c>
-      <c r="B42" t="s">
-        <v>37</v>
-      </c>
-      <c r="D42" t="s">
-        <v>86</v>
-      </c>
-      <c r="E42" t="s">
-        <v>78</v>
-      </c>
-      <c r="F42" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6">
-      <c r="A43">
-        <v>3</v>
-      </c>
-      <c r="B43" t="s">
-        <v>38</v>
-      </c>
-      <c r="D43" t="s">
-        <v>86</v>
-      </c>
-      <c r="E43" t="s">
-        <v>78</v>
-      </c>
-      <c r="F43" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6">
-      <c r="A44">
-        <v>3</v>
-      </c>
-      <c r="B44" t="s">
-        <v>39</v>
-      </c>
-      <c r="D44" t="s">
-        <v>86</v>
-      </c>
-      <c r="E44" t="s">
-        <v>98</v>
-      </c>
-      <c r="F44" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6">
-      <c r="A45">
-        <v>3</v>
-      </c>
-      <c r="B45" t="s">
-        <v>40</v>
-      </c>
-      <c r="D45" t="s">
-        <v>86</v>
-      </c>
-      <c r="E45" t="s">
-        <v>99</v>
-      </c>
-      <c r="F45" t="s">
-        <v>49</v>
+      <c r="F47" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1"/>
+    <hyperlink ref="D7" r:id="rId2"/>
+    <hyperlink ref="D13" r:id="rId3"/>
+    <hyperlink ref="D19" r:id="rId4"/>
+    <hyperlink ref="D25" r:id="rId5"/>
+    <hyperlink ref="D31" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>